<commit_message>
testing user and add some changes and fixing
</commit_message>
<xml_diff>
--- a/rtrw_terpadu_data_dictionary.xlsx
+++ b/rtrw_terpadu_data_dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\RTRW-Terpadu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2909E7E8-3203-4540-8F10-F6882F2EFCC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE343A0-763B-4C87-A016-111AA90CE187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="roles" sheetId="1" r:id="rId1"/>
@@ -856,6 +856,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1960,6 +1967,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.26953125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -2129,6 +2143,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.36328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -2329,6 +2350,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>